<commit_message>
fix: preserve branch area, facility and meal review metadata
</commit_message>
<xml_diff>
--- a/data/collections/osaka_branches_20261019/collection.xlsx
+++ b/data/collections/osaka_branches_20261019/collection.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="지점별 수집" sheetId="1" r:id="R5b321039f6c247e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기존 중복 확인" sheetId="2" r:id="Rae1962961a4e401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류·제외" sheetId="3" r:id="Re281e84ccfad4844"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="지점별 수집" sheetId="1" r:id="R20e46ff1ba654980"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기존 중복 확인" sheetId="2" r:id="Rc380c569482246db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류·제외" sheetId="3" r:id="Rd3c1a17c31554574"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -564,7 +564,7 @@
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
       <x:c r="I3" s="2" t="str">
-        <x:v>주소·시간은 출처 기준이고, 카테고리·세부 유형·표시 이름·검색 표기는 방문 목적에 따른 작업 분류예요.</x:v>
+        <x:v>권역은 임시 작업 분류예요. 시설 관계·끼니 역할·분류 ID 등 구조화 검토 항목은 branches.json과 README를 함께 확인해 주세요.</x:v>
       </x:c>
       <x:c r="J3" s="2"/>
       <x:c r="K3" s="2"/>
@@ -1849,7 +1849,7 @@
         <x:v>유니클로</x:v>
       </x:c>
       <x:c r="D26" s="13" t="str">
-        <x:v>유니클로 우메다점 (링크스)</x:v>
+        <x:v>유니클로 링크스 우메다점</x:v>
       </x:c>
       <x:c r="E26" s="13" t="str">
         <x:v>ユニクロ UMEDA</x:v>
@@ -1896,7 +1896,7 @@
       <x:c r="W26" s="20"/>
       <x:c r="X26" s="15"/>
       <x:c r="Y26" s="13" t="str">
-        <x:v>유니클로 우메다점 | 유니클로 링크스 우메다 | UNIQLO UMEDA</x:v>
+        <x:v>유니클로 우메다점 | 유니클로 링크스 우메다 | UNIQLO UMEDA | 유니클로 우메다점 (링크스)</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="115" customHeight="1">
@@ -2583,7 +2583,7 @@
         <x:v>베이프</x:v>
       </x:c>
       <x:c r="D38" s="13" t="str">
-        <x:v>베이프 꼼데가르송 오사카점</x:v>
+        <x:v>베이프 스토어 (꼼데가르송 오사카 내)</x:v>
       </x:c>
       <x:c r="E38" s="13" t="str">
         <x:v>BAPE STORE COMME DES GARCONS OSAKA</x:v>
@@ -2595,7 +2595,7 @@
         <x:v>쇼핑</x:v>
       </x:c>
       <x:c r="H38" s="13" t="str">
-        <x:v>스트리트 의류·협업 매장</x:v>
+        <x:v>스트리트 의류</x:v>
       </x:c>
       <x:c r="I38" s="13" t="str">
         <x:v>大阪府大阪市中央区南船場4-4-21</x:v>
@@ -3624,7 +3624,7 @@
         <x:v>JAM</x:v>
       </x:c>
       <x:c r="D55" s="13" t="str">
-        <x:v>빈티지 JAM 아메리카무라점</x:v>
+        <x:v>JAM 아메리카무라점</x:v>
       </x:c>
       <x:c r="E55" s="13" t="str">
         <x:v>古着屋JAM VINTAGE&amp;SELECT アメリカ村店</x:v>
@@ -3685,7 +3685,7 @@
         <x:v>JAM</x:v>
       </x:c>
       <x:c r="D56" s="13" t="str">
-        <x:v>빈티지 JAM 신사이바시점</x:v>
+        <x:v>JAM 신사이바시점</x:v>
       </x:c>
       <x:c r="E56" s="13" t="str">
         <x:v>古着屋JAM VINTAGE&amp;SELECT 心斎橋店</x:v>
@@ -3882,7 +3882,7 @@
         <x:v>식사</x:v>
       </x:c>
       <x:c r="H59" s="13" t="str">
-        <x:v>중화요리·부타만 / 식당</x:v>
+        <x:v>중화요리·부타만</x:v>
       </x:c>
       <x:c r="I59" s="13" t="str">
         <x:v>大阪府大阪市中央区難波3-6-3</x:v>
@@ -3943,7 +3943,7 @@
         <x:v>식사</x:v>
       </x:c>
       <x:c r="H60" s="13" t="str">
-        <x:v>중화요리·부타만 / 식당</x:v>
+        <x:v>중화요리·부타만</x:v>
       </x:c>
       <x:c r="I60" s="13" t="str">
         <x:v>大阪府大阪市中央区難波2 なんばウォーク1番街北通り-4</x:v>
@@ -4004,7 +4004,7 @@
         <x:v>식사</x:v>
       </x:c>
       <x:c r="H61" s="13" t="str">
-        <x:v>부타만·중화식품 / 포장 구매</x:v>
+        <x:v>부타만·중화식품</x:v>
       </x:c>
       <x:c r="I61" s="13" t="str">
         <x:v>大阪府大阪市中央区難波5-1-5 大阪高島屋B1F</x:v>
@@ -4312,7 +4312,7 @@
         <x:v>식사</x:v>
       </x:c>
       <x:c r="H66" s="13" t="str">
-        <x:v>타코야키·간식</x:v>
+        <x:v>타코야키</x:v>
       </x:c>
       <x:c r="I66" s="13" t="str">
         <x:v>大阪府大阪市中央区難波千日前11-19</x:v>
@@ -4373,7 +4373,7 @@
         <x:v>식사</x:v>
       </x:c>
       <x:c r="H67" s="13" t="str">
-        <x:v>타코야키·간식</x:v>
+        <x:v>타코야키</x:v>
       </x:c>
       <x:c r="I67" s="13" t="str">
         <x:v>大阪府大阪市中央区道頓堀1-6-7</x:v>
@@ -4957,7 +4957,7 @@
       <x:formula1>"신규 후보,보완,보류"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G10:G87">
-      <x:formula1>"쇼핑,식사,카페,명소,문화,자연,체험·오락,복합문화,미정"</x:formula1>
+      <x:formula1>"쇼핑,식사,카페,명소,문화,자연,체험·오락,미정"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="T10:T87">
       <x:formula1>"실내,야외,혼합,미확인"</x:formula1>
@@ -4965,7 +4965,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fb37c3b98474906"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d43bd5ddb74473"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5062,7 +5062,7 @@
         <x:v>이치란 도톤보리 별관</x:v>
       </x:c>
       <x:c r="E7" s="31" t="str">
-        <x:v>기존 별관 기록 보완. 본관과 별개 지점; 신규 중복 등록하지 않음.</x:v>
+        <x:v>표시 이름 유지. 기존 ID 보완 제안이며 자동 적용하지 않음.</x:v>
       </x:c>
       <x:c r="F7" s="31" t="str">
         <x:v>https://ichiran.com/shop/kinki/dotonbori-south/</x:v>
@@ -5082,7 +5082,7 @@
         <x:v>다이마루 신사이바시점 본관</x:v>
       </x:c>
       <x:c r="E8" s="31" t="str">
-        <x:v>기존 기록 보완. 신규 장소 수에 포함하지 않음. 같은 백화점 안의 개별 브랜드와 방문 범위를 구분.</x:v>
+        <x:v>이름 변경 제안: 다이마루 신사이바시점 → 다이마루 신사이바시점 본관. 검토 필요, 자동 적용하지 않음.</x:v>
       </x:c>
       <x:c r="F8" s="31" t="str">
         <x:v>https://www.daimaru.co.jp/shinsaibashi/hours.html</x:v>
@@ -5102,7 +5102,7 @@
         <x:v>한큐 우메다 본점</x:v>
       </x:c>
       <x:c r="E9" s="31" t="str">
-        <x:v>기존 기록 보완. 신규 장소 수에 포함하지 않음. 같은 백화점 안의 개별 브랜드와 방문 범위를 구분.</x:v>
+        <x:v>이름 변경 제안: 한큐 백화점 우메다 본점 → 한큐 우메다 본점. 검토 필요, 자동 적용하지 않음.</x:v>
       </x:c>
       <x:c r="F9" s="31" t="str">
         <x:v>https://www.hankyu-dept.co.jp/honten/map/index.html</x:v>
@@ -5119,7 +5119,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd42edaa02a6648e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R517e360caf5944d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5244,7 +5244,7 @@
         <x:v>2026-10-19T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="118" customHeight="1">
+    <x:row r="8" ht="155" customHeight="1">
       <x:c r="A8" s="31" t="str">
         <x:v>이치란 도톤보리 본관 (기존 기록)</x:v>
       </x:c>
@@ -5261,7 +5261,7 @@
         <x:v>기존 ID osm_node_2546559085 보존. 공식 목록에 없는 것만으로 폐업 확정하지 않음. 별관과 합치지 않음.</x:v>
       </x:c>
       <x:c r="F8" s="31" t="str">
-        <x:v>현재 운영 여부·정확한 지점·입구를 확인한 뒤 기존 기록 보완.</x:v>
+        <x:v>현재 운영 여부·정확한 지점·입구를 확인한 뒤 기존 ID를 유지하여 보완. 본관 동일성 확인 및 보류 해제 시 표시 이름을 이치란 도톤보리 본관으로 변경 제안하고 별도 검토.</x:v>
       </x:c>
       <x:c r="G8" s="31" t="str">
         <x:v>https://ichiran.com/shop/area-kinki.html</x:v>
@@ -5283,7 +5283,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d1a654144ea4ca5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2be0c86190014881"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>